<commit_message>
feat: add validated silver core pipeline
</commit_message>
<xml_diff>
--- a/docs/data_quality_rules.xlsx
+++ b/docs/data_quality_rules.xlsx
@@ -9,12 +9,18 @@
   <sheets>
     <sheet name="dq_rules" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="property_type_thresholds" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="profiling_baseline" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="count_field_profiling" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="expected_rule_hits" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="profiling_baseline" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="design_notes" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'dq_rules'!$A$1:$F$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'property_type_thresholds'!$A$1:$C$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'profiling_baseline'!$A$1:$C$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'dq_rules'!$A$1:$K$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'property_type_thresholds'!$A$1:$O$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'count_field_profiling'!$A$1:$R$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'expected_rule_hits'!$A$1:$G$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'profiling_baseline'!$A$1:$C$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'design_notes'!$A$1:$B$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,18 +454,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="65" customWidth="1" min="3" max="3"/>
+    <col width="57" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="65" customWidth="1" min="7" max="7"/>
+    <col width="65" customWidth="1" min="8" max="8"/>
+    <col width="43" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
+    <col width="65" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>rule_id</t>
@@ -467,7 +478,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>column</t>
+          <t>field</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -487,7 +498,32 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>field_validity_effect</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>action</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>affected_analytics</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>threshold_scope</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>rule_version</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>implementation_notes</t>
         </is>
       </c>
     </row>
@@ -499,17 +535,17 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>price</t>
+          <t>price_raw / price_vnd</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>price IS NULL</t>
+          <t>price_raw IS NULL OR TRIM(price_raw) = ''</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Giá bán bị thiếu</t>
+          <t>Thiếu giá đăng</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -519,7 +555,32 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Không dùng record này khi tính KPI liên quan đến giá</t>
+          <t>is_price_valid = false</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Giữ trong Silver Audit; không dùng cho KPI giá</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>price, price_per_m2</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>src01_silver_core_dq_v1</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Không loại khỏi KPI đếm tin đăng nếu KPI đó không cần giá.</t>
         </is>
       </c>
     </row>
@@ -531,17 +592,17 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>price</t>
+          <t>price_raw / price_vnd</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>price = 0</t>
+          <t>price_vnd &lt;= 0</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Giá bán bằng 0</t>
+          <t>Giá đăng không dương</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -551,7 +612,32 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Loại khỏi các bảng Gold phân tích giá</t>
+          <t>is_price_valid = false</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Giữ trong Silver Audit; loại khỏi KPI giá</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>price, price_per_m2</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>NON_POSITIVE</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>src01_silver_core_dq_v1</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>REJECTED chỉ áp dụng cho mục đích dùng giá, không phải xóa toàn bộ record.</t>
         </is>
       </c>
     </row>
@@ -563,17 +649,17 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>price</t>
+          <t>price_raw / price_vnd</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>TRY_CAST(price AS numeric) IS NULL</t>
+          <t>price_raw IS NOT NULL AND TRIM(price_raw) &lt;&gt; '' AND TRY_CAST(price_raw AS DECIMAL(20,0)) IS NULL</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Giá không chuyển được sang số</t>
+          <t>Giá có dữ liệu nhưng không chuyển được sang số</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -583,7 +669,32 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Loại khỏi Silver analytics</t>
+          <t>is_price_valid = false</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Giữ price_raw, đặt price_vnd = NULL; loại khỏi KPI giá</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>price, price_per_m2</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>CAST</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>src01_silver_core_dq_v1</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Điều kiện loại trừ NULL/blank nên không còn bắt trùng DQ01.</t>
         </is>
       </c>
     </row>
@@ -595,17 +706,17 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>area</t>
+          <t>area_m2</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>area IS NULL OR area &lt;= 0</t>
+          <t>area_m2 IS NULL OR area_m2 &lt;= 0</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Diện tích thiếu hoặc không hợp lệ</t>
+          <t>Diện tích thiếu hoặc không dương</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -615,7 +726,32 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Không thể tính price_per_m2</t>
+          <t>is_area_valid = false</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Giữ trong Silver Audit; không tính price_per_m2</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>area, price_per_m2</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>POSITIVE</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>src01_silver_core_dq_v1</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Record vẫn có thể dùng cho KPI không phụ thuộc diện tích.</t>
         </is>
       </c>
     </row>
@@ -627,17 +763,17 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>area</t>
+          <t>area_m2</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>area &gt; P99 theo property_type</t>
+          <t>area_m2 &gt; COALESCE(property_type_threshold.p99_area_m2, global_fallback.p99_area_m2)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Diện tích bất thường so với cùng loại BĐS</t>
+          <t>Diện tích lớn hơn P99 của cùng loại bất động sản</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -647,7 +783,32 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Giữ record nhưng đánh dấu để kiểm tra</t>
+          <t>Không tự động đổi is_area_valid</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Giữ giá trị và gắn cờ review; Gold sạch tự chọn có loại outlier hay không</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>area distribution, price_per_m2</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>P99_BY_PROPERTY_TYPE_WITH_GLOBAL_FALLBACK</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>src01_silver_core_dq_v1</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>P99 area được tính trên mọi area &gt; 0, không phụ thuộc price.</t>
         </is>
       </c>
     </row>
@@ -664,12 +825,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>price_per_m2 &gt; P99 theo property_type</t>
+          <t>unrounded(price_vnd / area_m2) &gt; COALESCE(property_type_threshold.p99_price_per_m2, global_fallback.p99_price_per_m2)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Giá/m² bất thường so với cùng loại BĐS</t>
+          <t>Giá đăng trên m² lớn hơn P99 của cùng loại bất động sản</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -679,7 +840,32 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Giữ record nhưng không dùng mặc định cho KPI sạch</t>
+          <t>Không tự động đổi is_price_valid/is_area_valid</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Giữ giá trị và gắn cờ review; mặc định loại khỏi KPI giá sạch</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>price_per_m2</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>P99_BY_PROPERTY_TYPE_WITH_GLOBAL_FALLBACK</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>src01_silver_core_dq_v1</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>So P99 bằng tỷ lệ chưa làm tròn như profiling; cột output price_per_m2 được lưu DECIMAL(24,2). Chỉ tính khi price &gt; 0 và area &gt; 0.</t>
         </is>
       </c>
     </row>
@@ -696,12 +882,12 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>province_name IS NULL OR TRIM(province_name)=''</t>
+          <t>province_name IS NULL OR TRIM(province_name) = ''</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Thiếu tỉnh/thành phố</t>
+          <t>Thiếu tỉnh/thành phố nguồn</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -711,7 +897,32 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Không thể phân tích theo vị trí</t>
+          <t>is_province_valid = false</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Giữ trong Silver Audit; không dùng cho KPI địa lý</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>province, district, ward geography</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>src01_silver_core_dq_v1</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Mapping mã hành chính thuộc Silver Enriched, không thuộc Core.</t>
         </is>
       </c>
     </row>
@@ -728,12 +939,12 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>district_name IS NULL</t>
+          <t>district_name IS NULL OR TRIM(district_name) = ''</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Thiếu quận/huyện</t>
+          <t>Thiếu quận/huyện nguồn</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -743,7 +954,32 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Vẫn giữ được phân tích cấp tỉnh</t>
+          <t>is_district_valid = false</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Giữ record; vẫn có thể dùng cho KPI cấp tỉnh</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>district, ward geography</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>src01_silver_core_dq_v1</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Không dùng row status toàn cục để loại khỏi KPI cấp tỉnh.</t>
         </is>
       </c>
     </row>
@@ -760,12 +996,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>ward_name IS NULL</t>
+          <t>ward_name IS NULL OR TRIM(ward_name) = ''</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Thiếu phường/xã</t>
+          <t>Thiếu phường/xã nguồn</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -775,7 +1011,32 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Vẫn giữ được phân tích cấp tỉnh/quận</t>
+          <t>is_ward_valid = false</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Giữ record; vẫn có thể dùng cho KPI cấp tỉnh/quận</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>ward geography</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>src01_silver_core_dq_v1</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Không dùng row status toàn cục để loại khỏi KPI cấp trên.</t>
         </is>
       </c>
     </row>
@@ -787,17 +1048,17 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>published_at</t>
+          <t>published_at_raw / published_at</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Không parse được timestamp</t>
+          <t>published_at_raw IS NULL OR TRIM(published_at_raw) = '' OR TRY_CAST(published_at_raw AS TIMESTAMP_NTZ) IS NULL</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Ngày đăng không hợp lệ</t>
+          <t>Ngày đăng thiếu hoặc không parse được</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -807,7 +1068,32 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Không thể phân tích theo thời gian</t>
+          <t>is_published_at_valid = false</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Giữ published_at_raw, đặt published_at = NULL; không dùng cho KPI thời gian</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>date, month, year trends</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>CAST</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>src01_silver_core_dq_v1</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Raw không có UTC offset; Silver v1 lưu TIMESTAMP_NTZ/source-local-naive và không tự gán UTC.</t>
         </is>
       </c>
     </row>
@@ -824,12 +1110,12 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Trùng khóa nội dung xác định</t>
+          <t>duplicate_rank &gt; 1 within duplicate_group_id built from source_id + source_name + all 19 raw business fields</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Bản ghi trùng lặp</t>
+          <t>Bản sao nội nguồn của cùng nhóm exact duplicate</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -839,7 +1125,32 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Giữ một bản ghi, loại bản sao</t>
+          <t>is_canonical = false</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Giữ mọi row trong Silver Audit; chỉ duplicate_rank = 1 vào analytical/canonical view</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>all aggregate counts and measures when canonical rows are required</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>EXACT_INTRA_SOURCE_DUPLICATE</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>src01_silver_core_dq_v1</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Dùng SHA-256 trên JSON null-safe có version của source_id, source_name và đủ 19 raw fields; không trim/cast trước hash. Baseline full-row: 36 nhóm, 50 dòng dư. Các bản sao exact trong cùng file không có physical row ID ổn định; canonical business row vẫn tương đương.</t>
         </is>
       </c>
     </row>
@@ -856,12 +1167,12 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Giá trị cực đoan/bất thường</t>
+          <t>floor_count IS NOT NULL AND floor_count &gt; COALESCE(property_type_threshold.p99_floor_count, 8)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Số tầng bất thường</t>
+          <t>Số tầng lớn hơn P99 theo loại BĐS</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -871,7 +1182,32 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Kiểm tra theo phân phối dữ liệu</t>
+          <t>Không tự động đổi tính hợp lệ của record</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Giữ record và giá trị; gắn cờ để review</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>floor_count</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>P99_BY_PROPERTY_TYPE; GLOBAL_FALLBACK=8</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>src01_silver_core_dq_v1</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Dùng quantile_disc và toán tử &gt;. SRC01 hiện có 0 giá trị âm/không nguyên; validator phải dừng nếu precondition này thay đổi trước khi cast INT.</t>
         </is>
       </c>
     </row>
@@ -888,12 +1224,12 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Giá trị cực đoan/bất thường</t>
+          <t>bedroom_count IS NOT NULL AND bedroom_count &gt; COALESCE(property_type_threshold.p99_bedroom_count, 14)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Số phòng ngủ bất thường</t>
+          <t>Số phòng ngủ lớn hơn P99 theo loại BĐS</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -903,7 +1239,32 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Kiểm tra theo phân phối dữ liệu</t>
+          <t>Không tự động đổi tính hợp lệ của record</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Giữ record và giá trị; gắn cờ để review</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>bedroom_count</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>P99_BY_PROPERTY_TYPE; GLOBAL_FALLBACK=14</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>src01_silver_core_dq_v1</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Dùng quantile_disc và toán tử &gt;. SRC01 hiện có 0 giá trị âm/không nguyên; validator phải dừng nếu precondition này thay đổi trước khi cast INT.</t>
         </is>
       </c>
     </row>
@@ -920,12 +1281,12 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Giá trị cực đoan/bất thường</t>
+          <t>bathroom_count IS NOT NULL AND bathroom_count &gt; COALESCE(property_type_threshold.p99_bathroom_count, 13)</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Số phòng tắm bất thường</t>
+          <t>Số phòng tắm lớn hơn P99 theo loại BĐS</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -935,12 +1296,37 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Kiểm tra theo phân phối dữ liệu</t>
+          <t>Không tự động đổi tính hợp lệ của record</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Giữ record và giá trị; gắn cờ để review</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>bathroom_count</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>P99_BY_PROPERTY_TYPE; GLOBAL_FALLBACK=13</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>src01_silver_core_dq_v1</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Dùng quantile_disc và toán tử &gt;. SRC01 hiện có 0 giá trị âm/không nguyên; validator phải dừng nếu precondition này thay đổi trước khi cast INT.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F15"/>
+  <autoFilter ref="A1:K15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -951,98 +1337,435 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="29" customWidth="1" min="12" max="12"/>
+    <col width="19" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>threshold_version</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>threshold_scope</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>property_type</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>total_rows</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>valid_area_rows</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>p99_area_m2</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>valid_price_per_m2_rows</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>p99_price_per_m2</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>floor_count_non_null_rows</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>p99_floor_count</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>bedroom_count_non_null_rows</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>p99_bedroom_count</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>bathroom_count_non_null_rows</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>p99_bathroom_count</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Nhà</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>550</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>735000000</v>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>GLOBAL_FALLBACK</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>__GLOBAL_FALLBACK__</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>3500744</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>3500740</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>2222</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>3224930</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>607692307.6923077</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>808762</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>1900383</v>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>1779770</v>
+      </c>
+      <c r="O2" s="2" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Đất</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>10363.2</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>347947900</v>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Biệt thự/Nhà liền kề</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>269782</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>269780</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>894.2520000000252</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>241579</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>625000000</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>135886</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>138989</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>131827</v>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
           <t>Căn hộ chung cư</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
-        <v>235</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>261864400</v>
+      <c r="E4" s="2" t="n">
+        <v>762800</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>762798</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>240</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>677895</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>261864406.779661</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>955</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>709883</v>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>682557</v>
+      </c>
+      <c r="O4" s="2" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Biệt thự/Nhà liền kề</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>900</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>625000000</v>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Nhà</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>1575536</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>1575536</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>544</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>1493988</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>735000000</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>649819</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>1026097</v>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>939093</v>
+      </c>
+      <c r="O5" s="2" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
           <t>Shophouse</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="E6" s="2" t="n">
+        <v>59860</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>59860</v>
+      </c>
+      <c r="G6" s="2" t="n">
         <v>535</v>
       </c>
-      <c r="C6" s="2" t="n">
-        <v>552310400</v>
+      <c r="H6" s="2" t="n">
+        <v>51717</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>552310374.8910201</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>20551</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>24734</v>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>25664</v>
+      </c>
+      <c r="O6" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Đất</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>832766</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>832766</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>10716.34999999998</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>759751</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>347947879.1170806</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>1551</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>680</v>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>629</v>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C6"/>
+  <autoFilter ref="A1:O7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1053,34 +1776,1573 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:R19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>metric</t>
+          <t>source_id</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>threshold_version</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>property_type</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>input_rows</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>non_null_rows</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>null_rows</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>zero_rows</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>negative_rows</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>non_integer_rows</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>min_value</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>p50</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>p95</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>p99_cont</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>p99_disc</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>max_value</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>recommended_review_threshold</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>bathroom_count</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>3500744</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>1779770</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>1720974</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="O2" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="P2" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q2" s="2" t="n">
+        <v>255</v>
+      </c>
+      <c r="R2" s="2" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Biệt thự/Nhà liền kề</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>bathroom_count</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>269782</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>131827</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>137955</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>9.740000000005239</v>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q3" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="R3" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Căn hộ chung cư</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>bathroom_count</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>762800</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>682557</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>80243</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="P4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q4" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="R4" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Nhà</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>bathroom_count</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>1575536</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>939093</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>636443</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="O5" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="P5" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q5" s="2" t="n">
+        <v>255</v>
+      </c>
+      <c r="R5" s="2" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Shophouse</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>bathroom_count</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>59860</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>25664</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>34196</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="O6" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="P6" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q6" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="R6" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Đất</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>bathroom_count</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>832766</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>629</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>832137</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q7" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="R7" s="2" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>bedroom_count</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>3500744</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>1900383</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>1600361</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="O8" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="P8" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q8" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="R8" s="2" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Biệt thự/Nhà liền kề</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>bedroom_count</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>269782</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>138989</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>130793</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="O9" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="P9" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q9" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="R9" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Căn hộ chung cư</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>bedroom_count</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>762800</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>709883</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>52917</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O10" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="P10" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q10" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="R10" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Nhà</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>bedroom_count</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>1575536</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>1026097</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>549439</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="O11" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="P11" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q11" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="R11" s="2" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Shophouse</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>bedroom_count</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>59860</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>24734</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>35126</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="O12" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="P12" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q12" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="R12" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Đất</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>bedroom_count</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>832766</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>680</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>832086</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="O13" s="2" t="n">
+        <v>18.42000000000007</v>
+      </c>
+      <c r="P13" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q13" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="R13" s="2" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>floor_count</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>3500744</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>808762</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>2691982</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="O14" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>255</v>
+      </c>
+      <c r="R14" s="2" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Biệt thự/Nhà liền kề</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>floor_count</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>269782</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>135886</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>133896</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="O15" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="P15" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q15" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="R15" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Căn hộ chung cư</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>floor_count</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>762800</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>955</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>761845</v>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="N16" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="O16" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="P16" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="Q16" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="R16" s="2" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Nhà</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>floor_count</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>1575536</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>649819</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>925717</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N17" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="O17" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="P17" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q17" s="2" t="n">
+        <v>255</v>
+      </c>
+      <c r="R17" s="2" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Shophouse</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>floor_count</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>59860</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>20551</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>39309</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="O18" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="P18" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q18" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="R18" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Đất</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>floor_count</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>832766</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>1551</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>831215</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N19" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="O19" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="P19" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q19" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="R19" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:R19"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>threshold_version</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>rule_id</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>expected_hit_rows</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>threshold_scope</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>DQ05</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>34807</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>P99_BY_PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>STRICT_GREATER_THAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>DQ06</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>price_per_m2</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>32219</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>P99_BY_PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>STRICT_GREATER_THAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>DQ12</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>floor_count</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>6511</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>P99_BY_PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>STRICT_GREATER_THAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>DQ13</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>bedroom_count</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>14530</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>P99_BY_PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>STRICT_GREATER_THAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>SRC01</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>src01_raw_20260904_p99_v1</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>DQ14</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>bathroom_count</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>11636</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>P99_BY_PROPERTY_TYPE</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>STRICT_GREATER_THAN</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G6"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
           <t>total_rows</t>
         </is>
       </c>
@@ -1089,7 +3351,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Tổng số bản ghi</t>
+          <t>Tổng record SRC01</t>
         </is>
       </c>
     </row>
@@ -1104,7 +3366,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Số bản ghi thiếu giá</t>
+          <t>Thiếu giá</t>
         </is>
       </c>
     </row>
@@ -1119,14 +3381,14 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Số bản ghi có giá bằng 0</t>
+          <t>Giá bằng 0</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>invalid_price</t>
+          <t>negative_price</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
@@ -1134,177 +3396,304 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Price không cast được sang số</t>
+          <t>Giá nhỏ hơn 0</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>null_area</t>
+          <t>invalid_non_null_price</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Số bản ghi thiếu diện tích</t>
+          <t>Giá có dữ liệu nhưng không cast được</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>duplicate_groups</t>
+          <t>null_area</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Số nhóm duplicate</t>
+          <t>Thiếu diện tích</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>duplicate_records</t>
+          <t>blank_name</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>50</v>
+        <v>1868</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Số bản ghi duplicate dư</t>
+          <t>Tên rỗng sau TRIM; đang là quyết định DQ mở</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>median_area</t>
+          <t>blank_description</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>80</v>
+        <v>1868</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Median diện tích toàn bộ dataset</t>
+          <t>Mô tả rỗng sau TRIM; đang là quyết định DQ mở</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>p99_area</t>
+          <t>exact_duplicate_groups</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>2222</v>
+        <v>36</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>P99 diện tích toàn bộ dataset</t>
+          <t>Nhóm exact duplicate theo DQ11</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>max_area</t>
+          <t>exact_duplicate_excess_rows</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>82000000</v>
+        <v>50</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Diện tích lớn nhất quan sát được</t>
+          <t>Số bản sao dư theo DQ11</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>median_price</t>
+          <t>published_at_with_utc_offset</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>7300000000</v>
+        <v>0</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Median giá</t>
+          <t>Không quan sát thấy UTC offset trong raw timestamp</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C12"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>decision_or_note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>document_status</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED_AND_VALIDATED</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>source_scope</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Chỉ SRC01 / Silver Listing Core; chưa bao gồm mapping location</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>condition_dialect</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Điều kiện trong workbook là Spark SQL-style pseudocode; code thực tế phải dùng PySpark expressions/type contract tương đương</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>retention</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Mọi 3,500,744 row được giữ trong Silver Audit; không drop âm thầm</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>status_precedence</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Nếu có REJECTED =&gt; dq_status=REJECTED; nếu không nhưng có REVIEW =&gt; REVIEW; còn lại VALID</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>gold_filtering</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Gold phải lọc theo is_canonical và field-validity/error-code liên quan KPI; không dùng một filter dq_status toàn cục</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>threshold_policy</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>DQ05/DQ06/DQ12-DQ14 dùng P99 theo property_type; chỉ dùng global fallback khi loại BĐS chưa có threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>threshold_execution</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Pipeline phải đọc đúng threshold version từ CSV; không tự tính lại bằng Spark vì thuật toán percentile có thể khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>outlier_meaning</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Vượt P99 là REVIEW, không chứng minh dữ liệu sai và không tự động null/drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>duplicate_policy</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>DQ11 chỉ dedup exact duplicate nội SRC01. Cross-source entity matching là bài toán riêng trong tương lai</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>timezone_contract</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>published_at không có offset; Silver v1 dùng TIMESTAMP_NTZ/source-local-naive và không tự gán UTC</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>p99_price</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>136000000000</v>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>P99 giá</t>
+          <t>candidate_dq15</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>DEFERRED_NOT_IMPLEMENTED: 1,868 row có name và description rỗng sau TRIM; DQ v1 chỉ gồm DQ01-DQ14</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>max_price</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>2.6597191e+16</v>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Giá lớn nhất quan sát được</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>median_price_per_m2</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>97777780</v>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Median giá/m²</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>p99_price_per_m2</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>607692300</v>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>P99 giá/m²</t>
+          <t>implementation_status</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED_AND_VALIDATED: src/silver/01_build_silver_core.py + 02_validate_silver_core.py</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C16"/>
+  <autoFilter ref="A1:B14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>